<commit_message>
Data Story Studio: map panels, hero titles and example geography
- Map (choropleth) panels, only when a dimension's values are places:
  countries by name or ISO code, and states/provinces for 9 countries.
  Detection reads values, not column names. Boundaries are bundled
  Natural Earth GeoJSON so exported reports render offline.
- Map regions filter the dashboard on click; maps can be switched to
  and from bar charts.
- Dashboard hero: short editorial title with the key finding as a
  line beneath it; long titles scale down.
- Example dataset: stores carry an Australian state, so the example
  shows a revenue-by-state map.
- Layout keeps the map in the story when the model leaves it out.

Co-Authored-By: Claude Code <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Data-Story-Studio/data/Example/stores.xlsx
+++ b/Data-Story-Studio/data/Example/stores.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="28">
   <si>
     <t>store_id</t>
   </si>
@@ -22,6 +22,9 @@
     <t>store_name</t>
   </si>
   <si>
+    <t>state</t>
+  </si>
+  <si>
     <t>area</t>
   </si>
   <si>
@@ -62,6 +65,24 @@
   </si>
   <si>
     <t>Harbour Quay</t>
+  </si>
+  <si>
+    <t>New South Wales</t>
+  </si>
+  <si>
+    <t>Victoria</t>
+  </si>
+  <si>
+    <t>Queensland</t>
+  </si>
+  <si>
+    <t>Western Australia</t>
+  </si>
+  <si>
+    <t>South Australia</t>
+  </si>
+  <si>
+    <t>Tasmania</t>
   </si>
   <si>
     <t>Metro</t>
@@ -408,10 +429,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:5">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -424,89 +445,110 @@
       <c r="D1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4">
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D5" t="s">
+        <v>24</v>
+      </c>
+      <c r="E5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" t="s">
+        <v>21</v>
+      </c>
+      <c r="D6" t="s">
+        <v>23</v>
+      </c>
+      <c r="E6" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7" t="s">
         <v>10</v>
       </c>
-      <c r="C2" t="s">
+      <c r="B7" t="s">
         <v>16</v>
       </c>
-      <c r="D2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4">
-      <c r="A3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D3" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4">
-      <c r="A4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C4" t="s">
-        <v>17</v>
-      </c>
-      <c r="D4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4">
-      <c r="A5" t="s">
-        <v>7</v>
-      </c>
-      <c r="B5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" t="s">
-        <v>17</v>
-      </c>
-      <c r="D5" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4">
-      <c r="A6" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6" t="s">
-        <v>14</v>
-      </c>
-      <c r="C6" t="s">
-        <v>16</v>
-      </c>
-      <c r="D6" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4">
-      <c r="A7" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" t="s">
-        <v>15</v>
-      </c>
       <c r="C7" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="D7" t="s">
-        <v>18</v>
+        <v>23</v>
+      </c>
+      <c r="E7" t="s">
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>